<commit_message>
Configure backend for Vercel deployment
</commit_message>
<xml_diff>
--- a/income_details.xlsx
+++ b/income_details.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,18 +413,62 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>one monthj</v>
+        <v>das</v>
       </c>
       <c r="B2">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="C2" s="1">
-        <v>46073.22928240741</v>
+        <v>46169.22928240741</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>bdfgd</v>
+      </c>
+      <c r="B3">
+        <v>800</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46156.22928240741</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fghfg</v>
+      </c>
+      <c r="B4">
+        <v>8787</v>
+      </c>
+      <c r="C4" s="1">
+        <v>46136.22928240741</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>dasd</v>
+      </c>
+      <c r="B5">
+        <v>499</v>
+      </c>
+      <c r="C5" s="1">
+        <v>46129.22928240741</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>thil hralhna</v>
+      </c>
+      <c r="B6">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="1">
+        <v>46109.22928240741</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>